<commit_message>
Grey address and step wires (replace purple), kit BOM with the grey spool
The book's address/step wire colour is now grey #7E848D (dark theme #8C939D):
signal colours, breadboard wire colours and swatches, project files and docs.
Kit BOM: Core Electronics ADA2983 grey spool replaces the RS purple reel.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EcTtXWgrYRRySNdyMDwmGB
</commit_message>
<xml_diff>
--- a/kit/PC-2_Kit_BOM.xlsx
+++ b/kit/PC-2_Kit_BOM.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1343" uniqueCount="701">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1340" uniqueCount="697">
   <si>
     <t xml:space="preserve">PC-2 breadboard kit: parts cost</t>
   </si>
@@ -678,10 +678,10 @@
     <t xml:space="preserve">W03</t>
   </si>
   <si>
-    <t xml:space="preserve">22 AWG solid-core wire, purple (m)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">addresses and step numbers (about 4.7 m); cut from a 30 m reel</t>
+    <t xml:space="preserve">22 AWG solid-core wire, grey, 25 ft (7.6 m) spool</t>
+  </si>
+  <si>
+    <t xml:space="preserve">addresses and step numbers (about 4.7 m)</t>
   </si>
   <si>
     <t xml:space="preserve">MAR, RAM, Control sequencer and others</t>
@@ -1860,45 +1860,42 @@
     <t xml:space="preserve">Adafruit solid-core wire spool, 25 ft, 22 AWG, orange. $10.20 inc GST; breaks 10+ 8.99, 50+ 8.81 ex GST. Recorded ex GST.</t>
   </si>
   <si>
+    <t xml:space="preserve">ADA2983</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://core-electronics.com.au/solid-core-wire-spool-25ft-22awg-gray.html</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Adafruit solid-core wire spool, 25 ft (7.6 m), 22 AWG, gray (Adafruit 2983). $9.95 inc GST; breaks 10+ 8.77, 50+ 8.59 ex GST. Recorded ex GST. Replaces the RS purple reel (owner decision 30 Oct: address and step wires are grey).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ADA2988</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4 local, 37 more in 8-12 days</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://core-electronics.com.au/solid-core-wire-spool-25ft-22awg-green.html</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Adafruit solid-core wire spool, 25 ft, 22 AWG, green. $8.35 inc GST; breaks 10+ 7.36, 50+ 7.21 ex GST. Recorded ex GST.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Adafruit 4090 (ADA4090)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">none local; supplier lead time</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://core-electronics.com.au/catalog/product/view/sku/ADA4090</t>
+  </si>
+  <si>
+    <t xml:space="preserve">USB-C downstream breakout; two 5.1 kOhm CC resistors ask the source for 5 V at up to 1.5 A; 8-pin 0.1 in header (GND, VBUS, SBU2, CC1, D-, D+, SBU1, CC2). $5.40 inc GST. Recorded ex GST.</t>
+  </si>
+  <si>
     <t xml:space="preserve">RS Components Australia</t>
   </si>
   <si>
-    <t xml:space="preserve">842-5387 / MPN 3051/1 VI005</t>
-  </si>
-  <si>
-    <t xml:space="preserve">46 (ships from another location)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://au.rs-online.com/web/p/hook-up-wire/8425387</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Alpha Wire 22 AWG solid (1/0.64 mm) PVC hook-up wire, purple, 30 m reel; prices per reel ex GST ($98.33 inc GST); breaks 50+ $88.29, 250+ $72.69. Qty per kit in metres. Alternative: Alpha 1561 VI005 (RS 277-8041, 100 ft); AUD price not read.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ADA2988</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4 local, 37 more in 8-12 days</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://core-electronics.com.au/solid-core-wire-spool-25ft-22awg-green.html</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Adafruit solid-core wire spool, 25 ft, 22 AWG, green. $8.35 inc GST; breaks 10+ 7.36, 50+ 7.21 ex GST. Recorded ex GST.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Adafruit 4090 (ADA4090)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">none local; supplier lead time</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://core-electronics.com.au/catalog/product/view/sku/ADA4090</t>
-  </si>
-  <si>
-    <t xml:space="preserve">USB-C downstream breakout; two 5.1 kOhm CC resistors ask the source for 5 V at up to 1.5 A; 8-pin 0.1 in header (GND, VBUS, SBU2, CC1, D-, D+, SBU1, CC2). $5.40 inc GST. Recorded ex GST.</t>
-  </si>
-  <si>
     <t xml:space="preserve">517-6770 / MPN RUEF110</t>
   </si>
   <si>
@@ -2064,19 +2061,10 @@
     <t xml:space="preserve">Wire</t>
   </si>
   <si>
-    <t xml:space="preserve">The Altronics wire is 24 AWG and is excluded from costing. Three SparkFun boxes hold 22.9 m of each colour (red, black, yellow, blue, green, white). PC-2 needs about 21.6 m of yellow (bus), 32 m of green (data), 4.7 m of purple, 3.8 m of orange and 3.0 m of pink (clock). No Australian supplier was found for pink solid-core 22 AWG wire, so the kit's white is used for the clock wires (the book says so on p. 29, in Table 1.4 and in Appendix C).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Add W02 (orange spool), W03 (5 m of purple cut from a 30 m RS reel) and W04 (two green spools). Cut the yellow and green wires from the cutting list first.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Purple wire price</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The purple reel (RS 842-5387, Alpha Wire 3051/1 VI005, $89.39 ex GST for 30 m) is the only Australian solid-core 22 AWG purple found; one reel covers six kits. The cheaper Alpha 1561 VI005 (RS 277-8041, 100 ft) has no AUD price on record.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Price to confirm: check RS 277-8041 and the Adafruit 2990 violet spool before the prototype order.</t>
+    <t xml:space="preserve">The Altronics wire is 24 AWG and is excluded from costing. Three SparkFun boxes hold 22.9 m of each colour (red, black, yellow, blue, green, white). PC-2 needs about 21.6 m of yellow (bus), 32 m of green (data), 4.7 m of grey (addresses and steps), 3.8 m of orange and 3.0 m of pink (clock). No Australian supplier was found for pink solid-core 22 AWG wire, so the kit's white is used for the clock wires (the book says so on p. 29, in Table 1.4 and in Appendix C).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Add W02 (orange spool), W03 (grey spool) and W04 (two green spools). Cut the yellow and green wires from the cutting list first.</t>
   </si>
   <si>
     <t xml:space="preserve">Kit prep: J1 header</t>
@@ -2088,10 +2076,10 @@
     <t xml:space="preserve">Kit preparation: solder the header to each J1 before packing (pins down, component side up), and test VBUS-GND with a USB-C supply. The book says J1 comes with its pins fitted.</t>
   </si>
   <si>
-    <t xml:space="preserve">Orange wire stock</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The orange spool (Core ADA2986) was out of stock on the day.</t>
+    <t xml:space="preserve">Orange and grey wire stock</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The orange and grey spools (Core ADA2986, ADA2983) were out of stock on the day.</t>
   </si>
   <si>
     <t xml:space="preserve">Order early or buy from another Adafruit reseller.</t>
@@ -2731,15 +2719,15 @@
       </c>
       <c r="B6" s="6" t="n">
         <f aca="false">BOM!H55</f>
-        <v>655.3066</v>
+        <v>566.9326</v>
       </c>
       <c r="C6" s="6" t="n">
         <f aca="false">BOM!I55</f>
-        <v>509.5845</v>
+        <v>499.5657</v>
       </c>
       <c r="D6" s="6" t="n">
         <f aca="false">BOM!J55</f>
-        <v>478.27793</v>
+        <v>471.011</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2748,15 +2736,15 @@
       </c>
       <c r="B7" s="7" t="n">
         <f aca="false">B6*B5</f>
-        <v>655.3066</v>
+        <v>566.9326</v>
       </c>
       <c r="C7" s="7" t="n">
         <f aca="false">C6*C5</f>
-        <v>5095.845</v>
+        <v>4995.657</v>
       </c>
       <c r="D7" s="7" t="n">
         <f aca="false">D6*D5</f>
-        <v>47827.793</v>
+        <v>47101.1</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2972,15 +2960,15 @@
       </c>
       <c r="B23" s="7" t="n">
         <f aca="false">SUMIFS(BOM!H2:H54,BOM!B2:B54,$A23)</f>
-        <v>357.709</v>
+        <v>269.335</v>
       </c>
       <c r="C23" s="7" t="n">
         <f aca="false">SUMIFS(BOM!I2:I54,BOM!B2:B54,$A23)</f>
-        <v>262.7218</v>
+        <v>252.703</v>
       </c>
       <c r="D23" s="7" t="n">
         <f aca="false">SUMIFS(BOM!J2:J54,BOM!B2:B54,$A23)</f>
-        <v>249.54193</v>
+        <v>242.275</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5465,7 +5453,7 @@
         <v>217</v>
       </c>
       <c r="E48" s="12" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F48" s="8" t="s">
         <v>218</v>
@@ -5476,23 +5464,23 @@
       </c>
       <c r="H48" s="7" t="n">
         <f aca="false">_xlfn.MINIFS(Prices!$W$2:$W$106,Prices!$A$2:$A$106,$A48,Prices!$L$2:$L$106,"Y",Prices!$W$2:$W$106,"&gt;0")</f>
-        <v>98.329</v>
+        <v>9.955</v>
       </c>
       <c r="I48" s="7" t="n">
         <f aca="false">_xlfn.MINIFS(Prices!$X$2:$X$106,Prices!$A$2:$A$106,$A48,Prices!$L$2:$L$106,"Y",Prices!$X$2:$X$106,"&gt;0")</f>
-        <v>19.6658</v>
+        <v>9.647</v>
       </c>
       <c r="J48" s="7" t="n">
         <f aca="false">_xlfn.MINIFS(Prices!$Y$2:$Y$106,Prices!$A$2:$A$106,$A48,Prices!$L$2:$L$106,"Y",Prices!$Y$2:$Y$106,"&gt;0")</f>
-        <v>16.71593</v>
+        <v>9.449</v>
       </c>
       <c r="K48" s="8" t="str">
         <f aca="false">IFERROR(INDEX(Prices!$B$2:$B$106,MATCH($A48&amp;"|"&amp;TEXT($H48,"0.0000")&amp;"|Y",Prices!$Z$2:$Z$106,0)),"none")</f>
-        <v>RS Components Australia</v>
+        <v>Core Electronics</v>
       </c>
       <c r="L48" s="8" t="str">
         <f aca="false">IFERROR(INDEX(Prices!$B$2:$B$106,MATCH($A48&amp;"|"&amp;TEXT($J48,"0.0000")&amp;"|Y",Prices!$AA$2:$AA$106,0)),"none")</f>
-        <v>RS Components Australia</v>
+        <v>Core Electronics</v>
       </c>
       <c r="M48" s="8" t="str">
         <f aca="false">IF($G48=0,"NO PRICE",IF($G48=1,"Single source",""))</f>
@@ -5791,15 +5779,15 @@
       </c>
       <c r="H55" s="13" t="n">
         <f aca="false">SUM(H2:H54)</f>
-        <v>655.3066</v>
+        <v>566.9326</v>
       </c>
       <c r="I55" s="13" t="n">
         <f aca="false">SUM(I2:I54)</f>
-        <v>509.5845</v>
+        <v>499.5657</v>
       </c>
       <c r="J55" s="13" t="n">
         <f aca="false">SUM(J2:J54)</f>
-        <v>478.27793</v>
+        <v>471.011</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14680,34 +14668,34 @@
         <v>215</v>
       </c>
       <c r="B96" s="8" t="s">
+        <v>284</v>
+      </c>
+      <c r="C96" s="8" t="s">
         <v>610</v>
       </c>
-      <c r="C96" s="8" t="s">
-        <v>611</v>
-      </c>
       <c r="D96" s="12" t="n">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="E96" s="14" t="n">
-        <v>89.39</v>
+        <v>9.05</v>
       </c>
       <c r="F96" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="G96" s="14" t="n">
+        <v>8.77</v>
+      </c>
+      <c r="H96" s="12" t="n">
         <v>50</v>
       </c>
-      <c r="G96" s="14" t="n">
-        <v>88.29</v>
-      </c>
-      <c r="H96" s="12" t="n">
-        <v>250</v>
-      </c>
       <c r="I96" s="14" t="n">
-        <v>72.69</v>
+        <v>8.59</v>
       </c>
       <c r="J96" s="12" t="s">
         <v>263</v>
       </c>
       <c r="K96" s="8" t="s">
-        <v>612</v>
+        <v>606</v>
       </c>
       <c r="L96" s="12" t="s">
         <v>265</v>
@@ -14716,14 +14704,14 @@
         <v>607</v>
       </c>
       <c r="N96" s="15" t="s">
-        <v>613</v>
+        <v>611</v>
       </c>
       <c r="O96" s="8" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="P96" s="8" t="n">
         <f aca="false">IFERROR(VLOOKUP($A96,BOM!$A$2:$E$54,5,0),0)</f>
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="Q96" s="8" t="n">
         <f aca="false">CEILING($P96*Assumptions!$B$4/$D96,1)</f>
@@ -14731,43 +14719,43 @@
       </c>
       <c r="R96" s="8" t="n">
         <f aca="false">CEILING($P96*Assumptions!$B$5/$D96,1)</f>
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="S96" s="8" t="n">
         <f aca="false">CEILING($P96*Assumptions!$B$6/$D96,1)</f>
-        <v>17</v>
+        <v>100</v>
       </c>
       <c r="T96" s="7" t="n">
         <f aca="false">IF(ISNUMBER($E96),IF(AND(ISNUMBER($I96),ISNUMBER($H96)),IF($H96&lt;=$Q96,$I96,IF(AND(ISNUMBER($G96),ISNUMBER($F96)),IF($F96&lt;=$Q96,$G96,$E96),$E96)),IF(AND(ISNUMBER($G96),ISNUMBER($F96)),IF($F96&lt;=$Q96,$G96,$E96),$E96))*(1+IF($J96="Y",0,Assumptions!$B$3)),"")</f>
-        <v>98.329</v>
+        <v>9.955</v>
       </c>
       <c r="U96" s="7" t="n">
         <f aca="false">IF(ISNUMBER($E96),IF(AND(ISNUMBER($I96),ISNUMBER($H96)),IF($H96&lt;=$R96,$I96,IF(AND(ISNUMBER($G96),ISNUMBER($F96)),IF($F96&lt;=$R96,$G96,$E96),$E96)),IF(AND(ISNUMBER($G96),ISNUMBER($F96)),IF($F96&lt;=$R96,$G96,$E96),$E96))*(1+IF($J96="Y",0,Assumptions!$B$3)),"")</f>
-        <v>98.329</v>
+        <v>9.647</v>
       </c>
       <c r="V96" s="7" t="n">
         <f aca="false">IF(ISNUMBER($E96),IF(AND(ISNUMBER($I96),ISNUMBER($H96)),IF($H96&lt;=$S96,$I96,IF(AND(ISNUMBER($G96),ISNUMBER($F96)),IF($F96&lt;=$S96,$G96,$E96),$E96)),IF(AND(ISNUMBER($G96),ISNUMBER($F96)),IF($F96&lt;=$S96,$G96,$E96),$E96))*(1+IF($J96="Y",0,Assumptions!$B$3)),"")</f>
-        <v>98.329</v>
+        <v>9.449</v>
       </c>
       <c r="W96" s="7" t="n">
         <f aca="false">IF(ISNUMBER($T96),$Q96*$T96/Assumptions!$B$4,"")</f>
-        <v>98.329</v>
+        <v>9.955</v>
       </c>
       <c r="X96" s="7" t="n">
         <f aca="false">IF(ISNUMBER($U96),$R96*$U96/Assumptions!$B$5,"")</f>
-        <v>19.6658</v>
+        <v>9.647</v>
       </c>
       <c r="Y96" s="7" t="n">
         <f aca="false">IF(ISNUMBER($V96),$S96*$V96/Assumptions!$B$6,"")</f>
-        <v>16.71593</v>
+        <v>9.449</v>
       </c>
       <c r="Z96" s="8" t="str">
         <f aca="false">$A96&amp;"|"&amp;IF(ISNUMBER($W96),TEXT($W96,"0.0000"),"x")&amp;"|"&amp;$L96</f>
-        <v>W03|98.3290|Y</v>
+        <v>W03|9.9550|Y</v>
       </c>
       <c r="AA96" s="8" t="str">
         <f aca="false">$A96&amp;"|"&amp;IF(ISNUMBER($Y96),TEXT($Y96,"0.0000"),"x")&amp;"|"&amp;$L96</f>
-        <v>W03|16.7159|Y</v>
+        <v>W03|9.4490|Y</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14778,7 +14766,7 @@
         <v>284</v>
       </c>
       <c r="C97" s="8" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
       <c r="D97" s="12" t="n">
         <v>1</v>
@@ -14802,7 +14790,7 @@
         <v>263</v>
       </c>
       <c r="K97" s="8" t="s">
-        <v>616</v>
+        <v>614</v>
       </c>
       <c r="L97" s="12" t="s">
         <v>265</v>
@@ -14811,10 +14799,10 @@
         <v>607</v>
       </c>
       <c r="N97" s="15" t="s">
-        <v>617</v>
+        <v>615</v>
       </c>
       <c r="O97" s="8" t="s">
-        <v>618</v>
+        <v>616</v>
       </c>
       <c r="P97" s="8" t="n">
         <f aca="false">IFERROR(VLOOKUP($A97,BOM!$A$2:$E$54,5,0),0)</f>
@@ -14873,7 +14861,7 @@
         <v>284</v>
       </c>
       <c r="C98" s="8" t="s">
-        <v>619</v>
+        <v>617</v>
       </c>
       <c r="D98" s="12" t="n">
         <v>1</v>
@@ -14897,7 +14885,7 @@
         <v>263</v>
       </c>
       <c r="K98" s="8" t="s">
-        <v>620</v>
+        <v>618</v>
       </c>
       <c r="L98" s="12" t="s">
         <v>265</v>
@@ -14906,10 +14894,10 @@
         <v>266</v>
       </c>
       <c r="N98" s="15" t="s">
-        <v>621</v>
+        <v>619</v>
       </c>
       <c r="O98" s="8" t="s">
-        <v>622</v>
+        <v>620</v>
       </c>
       <c r="P98" s="8" t="n">
         <f aca="false">IFERROR(VLOOKUP($A98,BOM!$A$2:$E$54,5,0),0)</f>
@@ -14965,10 +14953,10 @@
         <v>225</v>
       </c>
       <c r="B99" s="8" t="s">
-        <v>610</v>
+        <v>621</v>
       </c>
       <c r="C99" s="8" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="D99" s="12" t="n">
         <v>10</v>
@@ -14988,7 +14976,7 @@
         <v>263</v>
       </c>
       <c r="K99" s="8" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="L99" s="12" t="s">
         <v>265</v>
@@ -14997,10 +14985,10 @@
         <v>35</v>
       </c>
       <c r="N99" s="15" t="s">
+        <v>624</v>
+      </c>
+      <c r="O99" s="8" t="s">
         <v>625</v>
-      </c>
-      <c r="O99" s="8" t="s">
-        <v>626</v>
       </c>
       <c r="P99" s="8" t="n">
         <f aca="false">IFERROR(VLOOKUP($A99,BOM!$A$2:$E$54,5,0),0)</f>
@@ -15059,7 +15047,7 @@
         <v>292</v>
       </c>
       <c r="C100" s="8" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="D100" s="12" t="n">
         <v>1</v>
@@ -15083,7 +15071,7 @@
         <v>263</v>
       </c>
       <c r="K100" s="8" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="L100" s="12" t="s">
         <v>265</v>
@@ -15092,10 +15080,10 @@
         <v>35</v>
       </c>
       <c r="N100" s="15" t="s">
+        <v>628</v>
+      </c>
+      <c r="O100" s="8" t="s">
         <v>629</v>
-      </c>
-      <c r="O100" s="8" t="s">
-        <v>630</v>
       </c>
       <c r="P100" s="8" t="n">
         <f aca="false">IFERROR(VLOOKUP($A100,BOM!$A$2:$E$54,5,0),0)</f>
@@ -15154,7 +15142,7 @@
         <v>284</v>
       </c>
       <c r="C101" s="8" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="D101" s="12" t="n">
         <v>1</v>
@@ -15170,7 +15158,7 @@
         <v>265</v>
       </c>
       <c r="K101" s="8" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="L101" s="12" t="s">
         <v>265</v>
@@ -15179,10 +15167,10 @@
         <v>266</v>
       </c>
       <c r="N101" s="15" t="s">
+        <v>632</v>
+      </c>
+      <c r="O101" s="8" t="s">
         <v>633</v>
-      </c>
-      <c r="O101" s="8" t="s">
-        <v>634</v>
       </c>
       <c r="P101" s="8" t="n">
         <f aca="false">IFERROR(VLOOKUP($A101,BOM!$A$2:$E$54,5,0),0)</f>
@@ -15241,7 +15229,7 @@
         <v>261</v>
       </c>
       <c r="C102" s="8" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="D102" s="12" t="n">
         <v>1</v>
@@ -15257,7 +15245,7 @@
         <v>263</v>
       </c>
       <c r="K102" s="8" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="L102" s="12" t="s">
         <v>265</v>
@@ -15266,10 +15254,10 @@
         <v>266</v>
       </c>
       <c r="N102" s="15" t="s">
+        <v>636</v>
+      </c>
+      <c r="O102" s="8" t="s">
         <v>637</v>
-      </c>
-      <c r="O102" s="8" t="s">
-        <v>638</v>
       </c>
       <c r="P102" s="8" t="n">
         <f aca="false">IFERROR(VLOOKUP($A102,BOM!$A$2:$E$54,5,0),0)</f>
@@ -15328,7 +15316,7 @@
         <v>284</v>
       </c>
       <c r="C103" s="8" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="D103" s="12" t="n">
         <v>1</v>
@@ -15352,7 +15340,7 @@
         <v>263</v>
       </c>
       <c r="K103" s="8" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="L103" s="12" t="s">
         <v>265</v>
@@ -15361,10 +15349,10 @@
         <v>35</v>
       </c>
       <c r="N103" s="15" t="s">
+        <v>640</v>
+      </c>
+      <c r="O103" s="8" t="s">
         <v>641</v>
-      </c>
-      <c r="O103" s="8" t="s">
-        <v>642</v>
       </c>
       <c r="P103" s="8" t="n">
         <f aca="false">IFERROR(VLOOKUP($A103,BOM!$A$2:$E$54,5,0),0)</f>
@@ -15423,7 +15411,7 @@
         <v>514</v>
       </c>
       <c r="C104" s="8" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="D104" s="12" t="n">
         <v>1</v>
@@ -15452,10 +15440,10 @@
         <v>35</v>
       </c>
       <c r="N104" s="15" t="s">
+        <v>643</v>
+      </c>
+      <c r="O104" s="8" t="s">
         <v>644</v>
-      </c>
-      <c r="O104" s="8" t="s">
-        <v>645</v>
       </c>
       <c r="P104" s="8" t="n">
         <f aca="false">IFERROR(VLOOKUP($A104,BOM!$A$2:$E$54,5,0),0)</f>
@@ -15514,7 +15502,7 @@
         <v>284</v>
       </c>
       <c r="C105" s="8" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="D105" s="12" t="n">
         <v>1</v>
@@ -15530,7 +15518,7 @@
         <v>265</v>
       </c>
       <c r="K105" s="8" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
       <c r="L105" s="12" t="s">
         <v>265</v>
@@ -15539,10 +15527,10 @@
         <v>35</v>
       </c>
       <c r="N105" s="15" t="s">
+        <v>647</v>
+      </c>
+      <c r="O105" s="8" t="s">
         <v>648</v>
-      </c>
-      <c r="O105" s="8" t="s">
-        <v>649</v>
       </c>
       <c r="P105" s="8" t="n">
         <f aca="false">IFERROR(VLOOKUP($A105,BOM!$A$2:$E$54,5,0),0)</f>
@@ -15601,7 +15589,7 @@
         <v>261</v>
       </c>
       <c r="C106" s="8" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="D106" s="12" t="n">
         <v>1</v>
@@ -15625,7 +15613,7 @@
         <v>263</v>
       </c>
       <c r="K106" s="8" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
       <c r="L106" s="12" t="s">
         <v>265</v>
@@ -15634,7 +15622,7 @@
         <v>35</v>
       </c>
       <c r="N106" s="15" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="O106" s="8" t="s">
         <v>393</v>
@@ -15785,7 +15773,7 @@
     <hyperlink ref="N93" r:id="rId92" display="https://www.altronics.com.au/product/w2430-solid-core-05mm-6-colour-hobby-wire-pack"/>
     <hyperlink ref="N94" r:id="rId93" display="https://core-electronics.com.au/hook-up-wire-assortment-solid-core-22-awg.html"/>
     <hyperlink ref="N95" r:id="rId94" display="https://core-electronics.com.au/solid-core-wire-spool-25ft-22awg-orange.html"/>
-    <hyperlink ref="N96" r:id="rId95" display="https://au.rs-online.com/web/p/hook-up-wire/8425387"/>
+    <hyperlink ref="N96" r:id="rId95" display="https://core-electronics.com.au/solid-core-wire-spool-25ft-22awg-gray.html"/>
     <hyperlink ref="N97" r:id="rId96" display="https://core-electronics.com.au/solid-core-wire-spool-25ft-22awg-green.html"/>
     <hyperlink ref="N98" r:id="rId97" display="https://core-electronics.com.au/catalog/product/view/sku/ADA4090"/>
     <hyperlink ref="N99" r:id="rId98" display="https://au.rs-online.com/web/p/resettable-fuses/5176770"/>
@@ -15813,7 +15801,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
@@ -15822,178 +15810,167 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
+        <v>652</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>653</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="C1" s="3" t="s">
         <v>654</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>655</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="20" t="s">
+        <v>655</v>
+      </c>
+      <c r="B2" s="20" t="s">
         <v>656</v>
       </c>
-      <c r="B2" s="20" t="s">
+      <c r="C2" s="20" t="s">
         <v>657</v>
-      </c>
-      <c r="C2" s="20" t="s">
-        <v>658</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="20" t="s">
+        <v>658</v>
+      </c>
+      <c r="B3" s="20" t="s">
         <v>659</v>
       </c>
-      <c r="B3" s="20" t="s">
+      <c r="C3" s="20" t="s">
         <v>660</v>
-      </c>
-      <c r="C3" s="20" t="s">
-        <v>661</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="20" t="s">
+        <v>661</v>
+      </c>
+      <c r="B4" s="20" t="s">
         <v>662</v>
       </c>
-      <c r="B4" s="20" t="s">
+      <c r="C4" s="20" t="s">
         <v>663</v>
-      </c>
-      <c r="C4" s="20" t="s">
-        <v>664</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="20" t="s">
+        <v>664</v>
+      </c>
+      <c r="B5" s="20" t="s">
         <v>665</v>
       </c>
-      <c r="B5" s="20" t="s">
+      <c r="C5" s="20" t="s">
         <v>666</v>
-      </c>
-      <c r="C5" s="20" t="s">
-        <v>667</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="20" t="s">
+        <v>667</v>
+      </c>
+      <c r="B6" s="20" t="s">
         <v>668</v>
       </c>
-      <c r="B6" s="20" t="s">
+      <c r="C6" s="20" t="s">
         <v>669</v>
-      </c>
-      <c r="C6" s="20" t="s">
-        <v>670</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="20" t="s">
+        <v>670</v>
+      </c>
+      <c r="B7" s="20" t="s">
         <v>671</v>
       </c>
-      <c r="B7" s="20" t="s">
+      <c r="C7" s="20" t="s">
         <v>672</v>
-      </c>
-      <c r="C7" s="20" t="s">
-        <v>673</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="20" t="s">
+        <v>673</v>
+      </c>
+      <c r="B8" s="20" t="s">
         <v>674</v>
       </c>
-      <c r="B8" s="20" t="s">
+      <c r="C8" s="20" t="s">
         <v>675</v>
-      </c>
-      <c r="C8" s="20" t="s">
-        <v>676</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="90.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="20" t="s">
+        <v>676</v>
+      </c>
+      <c r="B9" s="20" t="s">
         <v>677</v>
       </c>
-      <c r="B9" s="20" t="s">
+      <c r="C9" s="20" t="s">
         <v>678</v>
       </c>
-      <c r="C9" s="20" t="s">
+    </row>
+    <row r="10" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="20" t="s">
         <v>679</v>
       </c>
-    </row>
-    <row r="10" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="20" t="s">
+      <c r="B10" s="20" t="s">
         <v>680</v>
       </c>
-      <c r="B10" s="20" t="s">
+      <c r="C10" s="20" t="s">
         <v>681</v>
       </c>
-      <c r="C10" s="20" t="s">
+    </row>
+    <row r="11" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="20" t="s">
         <v>682</v>
       </c>
-    </row>
-    <row r="11" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="20" t="s">
+      <c r="B11" s="20" t="s">
         <v>683</v>
       </c>
-      <c r="B11" s="20" t="s">
+      <c r="C11" s="20" t="s">
         <v>684</v>
       </c>
-      <c r="C11" s="20" t="s">
+    </row>
+    <row r="12" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="20" t="s">
         <v>685</v>
       </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="20" t="s">
+      <c r="B12" s="20" t="s">
         <v>686</v>
       </c>
-      <c r="B12" s="20" t="s">
+      <c r="C12" s="20" t="s">
         <v>687</v>
-      </c>
-      <c r="C12" s="20" t="s">
-        <v>688</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="20" t="s">
+        <v>688</v>
+      </c>
+      <c r="B13" s="20" t="s">
         <v>689</v>
       </c>
-      <c r="B13" s="20" t="s">
+      <c r="C13" s="20" t="s">
         <v>690</v>
       </c>
-      <c r="C13" s="20" t="s">
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="20" t="s">
         <v>691</v>
       </c>
-    </row>
-    <row r="14" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="20" t="s">
+      <c r="B14" s="20" t="s">
         <v>692</v>
       </c>
-      <c r="B14" s="20" t="s">
+      <c r="C14" s="20" t="s">
         <v>693</v>
       </c>
-      <c r="C14" s="20" t="s">
+    </row>
+    <row r="15" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="20" t="s">
         <v>694</v>
       </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="20" t="s">
+      <c r="B15" s="20" t="s">
         <v>695</v>
       </c>
-      <c r="B15" s="20" t="s">
+      <c r="C15" s="20" t="s">
         <v>696</v>
-      </c>
-      <c r="C15" s="20" t="s">
-        <v>697</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="20" t="s">
-        <v>698</v>
-      </c>
-      <c r="B16" s="20" t="s">
-        <v>699</v>
-      </c>
-      <c r="C16" s="20" t="s">
-        <v>700</v>
       </c>
     </row>
   </sheetData>

</xml_diff>